<commit_message>
fix(mountain-map): update V8 tier pipeline
</commit_message>
<xml_diff>
--- a/scripts/mountain_map/construct_table.xlsx
+++ b/scripts/mountain_map/construct_table.xlsx
@@ -3791,7 +3791,7 @@
       </c>
       <c r="E3" s="5" t="inlineStr">
         <is>
-          <t>AST then engine bytecode (e.g. V8 Ignition bytecode)</t>
+          <t>AST then engine bytecode/baseline/JIT tiers (e.g. V8 Ignition bytecode, Sparkplug, Maglev, TurboFan)</t>
         </is>
       </c>
       <c r="F3" s="5" t="inlineStr">
@@ -3801,7 +3801,7 @@
       </c>
       <c r="G3" s="5" t="inlineStr">
         <is>
-          <t>The engine (e.g. V8) parses source to an AST, Ignition compiles it to bytecode and interprets it, and TurboFan JIT-compiles hot functions to native code.</t>
+          <t>The engine (e.g. V8) parses source to an AST, Ignition compiles it to bytecode and interprets it, Sparkplug baseline-compiles hot code, Maglev optimizes suitable hot functions, and TurboFan handles higher-tier optimizing JIT compilation.</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
fix(mountain-map): update V8 tier pipeline (#2385)
</commit_message>
<xml_diff>
--- a/scripts/mountain_map/construct_table.xlsx
+++ b/scripts/mountain_map/construct_table.xlsx
@@ -3791,7 +3791,7 @@
       </c>
       <c r="E3" s="5" t="inlineStr">
         <is>
-          <t>AST then engine bytecode (e.g. V8 Ignition bytecode)</t>
+          <t>AST then engine bytecode/baseline/JIT tiers (e.g. V8 Ignition bytecode, Sparkplug, Maglev, TurboFan)</t>
         </is>
       </c>
       <c r="F3" s="5" t="inlineStr">
@@ -3801,7 +3801,7 @@
       </c>
       <c r="G3" s="5" t="inlineStr">
         <is>
-          <t>The engine (e.g. V8) parses source to an AST, Ignition compiles it to bytecode and interprets it, and TurboFan JIT-compiles hot functions to native code.</t>
+          <t>The engine (e.g. V8) parses source to an AST, Ignition compiles it to bytecode and interprets it, Sparkplug baseline-compiles hot code, Maglev optimizes suitable hot functions, and TurboFan handles higher-tier optimizing JIT compilation.</t>
         </is>
       </c>
     </row>

</xml_diff>